<commit_message>
fix: Atualiza script de geracao e estrutura de relatorios v2.0
</commit_message>
<xml_diff>
--- a/outputs/dashboard_quimioinformatica_v2.xlsx
+++ b/outputs/dashboard_quimioinformatica_v2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,183 +424,116 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>CID</t>
+          <t>SMILES</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>SMILES</t>
+          <t>Origem</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Origem</t>
+          <t>Peso_Molecular</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Unidades</t>
+          <t>LogP</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Limitacoes</t>
+          <t>TPSA</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Peso_Molecular_g_mol</t>
+          <t>Rotatable_Bonds</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>LogP</t>
+          <t>QED</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>TPSA_A2</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Rotatable_Bonds</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>QED_Score</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Veber_Aprovado</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Origem_Calculo</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Limitacoes_ADMET</t>
+          <t>Regra_Veber</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Aspirin</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2244</v>
+          <t>Aspirina</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CC(=O)OC1=CC=CC=C1C(=O)O</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>PubChem PUG REST</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Adimensional / Padrão SMILES</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>SMILES canônico pode omitir estereoquímica complexa</t>
-        </is>
+          <t>PubChem</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>180.16</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F2" t="n">
+        <v>63.6</v>
       </c>
       <c r="G2" t="n">
-        <v>180.159</v>
+        <v>2</v>
       </c>
       <c r="H2" t="n">
-        <v>1.3101</v>
-      </c>
-      <c r="I2" t="n">
-        <v>63.60000000000001</v>
-      </c>
-      <c r="J2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.5501217966938848</v>
-      </c>
-      <c r="L2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>RDKit Descriptors</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Estimativas in silico baseadas em topologia molecular</t>
+        <v>0.55</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Caffeine</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2519</v>
+          <t>Cafeína</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CN1C=NC2=C1C(=O)N(C(=O)N2C)C</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CN1C=NC2=C1C(=O)N(C(=O)N2C)C</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>PubChem PUG REST</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Adimensional / Padrão SMILES</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>SMILES canônico pode omitir estereoquímica complexa</t>
-        </is>
+          <t>PubChem</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>194.19</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="F3" t="n">
+        <v>61.82</v>
       </c>
       <c r="G3" t="n">
-        <v>194.194</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>-1.0293</v>
-      </c>
-      <c r="I3" t="n">
-        <v>61.82</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.5384628262372215</v>
-      </c>
-      <c r="L3" t="b">
-        <v>1</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>RDKit Descriptors</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Estimativas in silico baseadas em topologia molecular</t>
+        <v>0.54</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
         </is>
       </c>
     </row>
@@ -610,55 +543,34 @@
           <t>Paracetamol</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>1983</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CC(=O)NC1=CC=C(O)C=C1</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CC(=O)NC1=CC=C(C=C1)O</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>PubChem PUG REST</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Adimensional / Padrão SMILES</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>SMILES canônico pode omitir estereoquímica complexa</t>
-        </is>
+          <t>PubChem</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>151.16</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F4" t="n">
+        <v>49.33</v>
       </c>
       <c r="G4" t="n">
-        <v>151.165</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>1.3506</v>
-      </c>
-      <c r="I4" t="n">
-        <v>49.33</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.5950261967780848</v>
-      </c>
-      <c r="L4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>RDKit Descriptors</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Estimativas in silico baseadas em topologia molecular</t>
+        <v>0.59</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Corrige intervalos das formulas de media no dashboard excel
</commit_message>
<xml_diff>
--- a/outputs/dashboard_quimioinformatica_v2.xlsx
+++ b/outputs/dashboard_quimioinformatica_v2.xlsx
@@ -237,12 +237,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard Executivo'!$B$10:$B$11</f>
+              <f>'Dashboard Executivo'!$B$10:$B$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard Executivo'!$C$10:$C$11</f>
+              <f>'Dashboard Executivo'!$C$10:$C$12</f>
             </numRef>
           </val>
         </ser>
@@ -676,12 +676,12 @@
       </c>
       <c r="C5" s="3" t="n"/>
       <c r="E5" s="5">
-        <f>AVERAGE(C9:C11)</f>
+        <f>AVERAGE(C10:C12)</f>
         <v/>
       </c>
       <c r="F5" s="3" t="n"/>
       <c r="H5" s="5">
-        <f>AVERAGE(D9:D11)</f>
+        <f>AVERAGE(D10:D12)</f>
         <v/>
       </c>
       <c r="I5" s="3" t="n"/>

</xml_diff>